<commit_message>
Berechne Systemname für Veranstaltungen aus Formulargruppe
Systemname ist mit der Sektion Trier abgesprochen: "<Jahr>
<Formulargruppe> <MonatTag> <Formular-Titel>". Der Titel bleibt eine
1:1-Kopie von "Bezeichnung/Titel".
</commit_message>
<xml_diff>
--- a/tests/fixtures/expected/veranstaltungen_tr.xlsx
+++ b/tests/fixtures/expected/veranstaltungen_tr.xlsx
@@ -556,7 +556,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2606WANFeierabendwanderung</t>
+          <t>26 Sonntagswanderung 0605 Feierabendwanderung</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -613,7 +613,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2606MTBFeierabendrundeMTB</t>
+          <t>26 Mountainbike 0612 Feierabendrunde MTB</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">

</xml_diff>